<commit_message>
Update trade logging to use lots and reflect in app views
Modify TradeBook.tsx to accept 'lots' and calculate actual quantity based on segment lot sizes. Update App.tsx to fetch and merge local trades from the API with Google Sheets data, making Trade Book entries visible in the Calendar and Dashboard.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 40f07ba7-651d-4579-8db9-38d55b18da28
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 157dba19-b3a7-4df6-846b-dd0e30f79901
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/06bd7d99-15c6-498d-9883-42f1906638af/40f07ba7-651d-4579-8db9-38d55b18da28/SLhgygE
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/server/trades.xlsx
+++ b/server/trades.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,9 +446,56 @@
         <v>Missed Profits</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>1-Jun</v>
+      </c>
+      <c r="D2" t="str">
+        <v>BankniftyPE</v>
+      </c>
+      <c r="E2">
+        <v>120</v>
+      </c>
+      <c r="F2">
+        <v>522.8</v>
+      </c>
+      <c r="G2">
+        <v>496.85</v>
+      </c>
+      <c r="H2">
+        <v>-25.949999999999932</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>3263.999999999992</v>
+      </c>
+      <c r="K2">
+        <v>150</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2">
+        <v>-3263.999999999992</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply a dark theme to the Trade Book and fix the refresh functionality
Rewrite the TradeBook component with dark theme styling and ensure the refresh button correctly triggers data refetching for both Google Sheets and local trades.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 40f07ba7-651d-4579-8db9-38d55b18da28
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ba813c9b-2355-48d4-9459-485700a0fb7e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/06bd7d99-15c6-498d-9883-42f1906638af/40f07ba7-651d-4579-8db9-38d55b18da28/0JQbSGx
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/server/trades.xlsx
+++ b/server/trades.xlsx
@@ -466,16 +466,16 @@
         <v>522.8</v>
       </c>
       <c r="G2">
-        <v>496.83</v>
+        <v>496.85</v>
       </c>
       <c r="H2">
-        <v>-25.96999999999997</v>
+        <v>-25.949999999999932</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>3266.3999999999965</v>
+        <v>3263.999999999992</v>
       </c>
       <c r="K2">
         <v>150</v>
@@ -487,7 +487,7 @@
         <v/>
       </c>
       <c r="N2">
-        <v>-3266.3999999999965</v>
+        <v>-3263.999999999992</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
Restore the dark theme for the trade book with updated segments
Reverts the TradeBook component to its dark theme aesthetic, incorporating the latest Excel-based segments and their associated lot sizes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 40f07ba7-651d-4579-8db9-38d55b18da28
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b86a15a1-ca79-4286-973e-6f6e736f30ca
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/06bd7d99-15c6-498d-9883-42f1906638af/40f07ba7-651d-4579-8db9-38d55b18da28/P1ikjl7
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/server/trades.xlsx
+++ b/server/trades.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,56 +446,9 @@
         <v>Missed Profits</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v>1-Jun</v>
-      </c>
-      <c r="D2" t="str">
-        <v>BankniftyPE</v>
-      </c>
-      <c r="E2">
-        <v>120</v>
-      </c>
-      <c r="F2">
-        <v>522.8</v>
-      </c>
-      <c r="G2">
-        <v>496.85</v>
-      </c>
-      <c r="H2">
-        <v>-25.949999999999932</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>3263.999999999992</v>
-      </c>
-      <c r="K2">
-        <v>150</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2">
-        <v>-3263.999999999992</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update trade book functionality and calendar view
Implement auto-refresh for trade book data, make refresh button visible on all tabs, and adjust calendar lot values for June 2026 onwards.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: feb426c7-5b2e-45b4-a696-dbb72e6c2bfb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 202007a7-47e0-45e8-81c3-bb693b92fdb3
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e42c11dd-cdf9-45e0-836a-4b63cd3b9eec/feb426c7-5b2e-45b4-a696-dbb72e6c2bfb/EfnrDoI
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/server/trades.xlsx
+++ b/server/trades.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,9 +446,56 @@
         <v>Missed Profits</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>01-06-2026</v>
+      </c>
+      <c r="D2" t="str">
+        <v>BankniftyPE</v>
+      </c>
+      <c r="E2">
+        <v>120</v>
+      </c>
+      <c r="F2">
+        <v>522.8</v>
+      </c>
+      <c r="G2">
+        <v>496.85</v>
+      </c>
+      <c r="H2">
+        <v>-25.949999999999932</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>3243.999999999992</v>
+      </c>
+      <c r="K2">
+        <v>130</v>
+      </c>
+      <c r="L2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2">
+        <v>-3243.999999999992</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Preserve exact numeric precision during data migration and updates
Remove Math.round from lot quantity calculations in TradeBook.tsx and ensure all numeric data is migrated and stored without loss of precision.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: c81873ae-1475-49ad-a48c-08261a308bad
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 18664498-9a42-4e94-92b6-e559de4e8ea0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/524b837a-5475-4f48-b8c0-de4e7391897c/c81873ae-1475-49ad-a48c-08261a308bad/M25oyT5
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/server/trades.xlsx
+++ b/server/trades.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O221"/>
+  <dimension ref="A1:O220"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,7 +454,7 @@
         <v/>
       </c>
       <c r="C2" t="str">
-        <v>14-10-2025</v>
+        <v>14-10-2024</v>
       </c>
       <c r="D2" t="str">
         <v>BankniftyPE</v>
@@ -478,7 +478,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L2" t="str">
         <v>Yes</v>
@@ -501,7 +501,7 @@
         <v/>
       </c>
       <c r="C3" t="str">
-        <v>15-10-2025</v>
+        <v>15-10-2024</v>
       </c>
       <c r="D3" t="str">
         <v>NiftyCE</v>
@@ -525,7 +525,7 @@
         <v>-2254</v>
       </c>
       <c r="K3">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L3" t="str">
         <v>Yes</v>
@@ -548,7 +548,7 @@
         <v/>
       </c>
       <c r="C4" t="str">
-        <v>15-10-2025</v>
+        <v>15-10-2024</v>
       </c>
       <c r="D4" t="str">
         <v>NiftyCE</v>
@@ -572,7 +572,7 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L4" t="str">
         <v>Yes</v>
@@ -595,7 +595,7 @@
         <v/>
       </c>
       <c r="C5" t="str">
-        <v>15-10-2025</v>
+        <v>15-10-2024</v>
       </c>
       <c r="D5" t="str">
         <v>BankniftyCE</v>
@@ -619,7 +619,7 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L5" t="str">
         <v>Yes</v>
@@ -642,7 +642,7 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <v>17-10-2025</v>
+        <v>17-10-2024</v>
       </c>
       <c r="D6" t="str">
         <v>Sensex CE</v>
@@ -666,7 +666,7 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L6" t="str">
         <v>Yes</v>
@@ -689,7 +689,7 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>17-10-2025</v>
+        <v>17-10-2024</v>
       </c>
       <c r="D7" t="str">
         <v>BankniftyCE</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L7" t="str">
         <v>Yes</v>
@@ -736,7 +736,7 @@
         <v/>
       </c>
       <c r="C8" t="str">
-        <v>17-10-2025</v>
+        <v>17-10-2024</v>
       </c>
       <c r="D8" t="str">
         <v>NiftyCE</v>
@@ -760,7 +760,7 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L8" t="str">
         <v>Yes</v>
@@ -783,7 +783,7 @@
         <v/>
       </c>
       <c r="C9" t="str">
-        <v>17-10-2025</v>
+        <v>17-10-2024</v>
       </c>
       <c r="D9" t="str">
         <v>BankniftyPE</v>
@@ -807,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L9" t="str">
         <v>Yes</v>
@@ -830,7 +830,7 @@
         <v/>
       </c>
       <c r="C10" t="str">
-        <v>20-10-2025</v>
+        <v>20-10-2024</v>
       </c>
       <c r="D10" t="str">
         <v>BankniftyCE</v>
@@ -854,7 +854,7 @@
         <v>-994</v>
       </c>
       <c r="K10">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L10" t="str">
         <v>Yes</v>
@@ -877,7 +877,7 @@
         <v/>
       </c>
       <c r="C11" t="str">
-        <v>23-10-2025</v>
+        <v>23-10-2024</v>
       </c>
       <c r="D11" t="str">
         <v>Sensex PE</v>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L11" t="str">
         <v>Yes</v>
@@ -924,7 +924,7 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>23-10-2025</v>
+        <v>23-10-2024</v>
       </c>
       <c r="D12" t="str">
         <v>Sensex PE</v>
@@ -948,7 +948,7 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L12" t="str">
         <v>Yes</v>
@@ -971,7 +971,7 @@
         <v/>
       </c>
       <c r="C13" t="str">
-        <v>23-10-2025</v>
+        <v>23-10-2024</v>
       </c>
       <c r="D13" t="str">
         <v>NiftyCE</v>
@@ -995,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L13" t="str">
         <v>Yes</v>
@@ -1018,7 +1018,7 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <v>24-10-2025</v>
+        <v>24-10-2024</v>
       </c>
       <c r="D14" t="str">
         <v>BankniftyPE</v>
@@ -1042,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L14" t="str">
         <v>Yes</v>
@@ -1065,7 +1065,7 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>27-10-2025</v>
+        <v>27-10-2024</v>
       </c>
       <c r="D15" t="str">
         <v>BankniftyCE</v>
@@ -1089,7 +1089,7 @@
         <v>-2107</v>
       </c>
       <c r="K15">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L15" t="str">
         <v>Yes</v>
@@ -1112,7 +1112,7 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>27-10-2025</v>
+        <v>27-10-2024</v>
       </c>
       <c r="D16" t="str">
         <v>Sensex CE</v>
@@ -1136,7 +1136,7 @@
         <v>-1501</v>
       </c>
       <c r="K16">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L16" t="str">
         <v>yes</v>
@@ -1159,7 +1159,7 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>29-10-2025</v>
+        <v>29-10-2024</v>
       </c>
       <c r="D17" t="str">
         <v>NiftyCE</v>
@@ -1183,7 +1183,7 @@
         <v>-1849</v>
       </c>
       <c r="K17">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L17" t="str">
         <v>yes</v>
@@ -1206,7 +1206,7 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>29-10-2025</v>
+        <v>29-10-2024</v>
       </c>
       <c r="D18" t="str">
         <v>BankniftyCE</v>
@@ -1230,7 +1230,7 @@
         <v>-693</v>
       </c>
       <c r="K18">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L18" t="str">
         <v>yes</v>
@@ -1253,7 +1253,7 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>30-10-2025</v>
+        <v>30-10-2024</v>
       </c>
       <c r="D19" t="str">
         <v>Sensex PE</v>
@@ -1277,7 +1277,7 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L19" t="str">
         <v>No</v>
@@ -1300,7 +1300,7 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>04-11-2025</v>
+        <v>04-11-2024</v>
       </c>
       <c r="D20" t="str">
         <v>NiftyPE</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="K20">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L20" t="str">
         <v>Yes</v>
@@ -1347,7 +1347,7 @@
         <v/>
       </c>
       <c r="C21" t="str">
-        <v>06-11-2025</v>
+        <v>06-11-2024</v>
       </c>
       <c r="D21" t="str">
         <v>BankniftyPE</v>
@@ -1371,7 +1371,7 @@
         <v>-2849</v>
       </c>
       <c r="K21">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L21" t="str">
         <v>Yes</v>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="C22" t="str">
-        <v>07-11-2025</v>
+        <v>07-11-2024</v>
       </c>
       <c r="D22" t="str">
         <v>NiftyPE</v>
@@ -1418,7 +1418,7 @@
         <v>-3908</v>
       </c>
       <c r="K22">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L22" t="str">
         <v>yes</v>
@@ -1441,7 +1441,7 @@
         <v/>
       </c>
       <c r="C23" t="str">
-        <v>07-11-2025</v>
+        <v>07-11-2024</v>
       </c>
       <c r="D23" t="str">
         <v>Sensex PE</v>
@@ -1465,7 +1465,7 @@
         <v>-3834</v>
       </c>
       <c r="K23">
-        <v>-40</v>
+        <v>40</v>
       </c>
       <c r="L23" t="str">
         <v>Yes</v>
@@ -1488,7 +1488,7 @@
         <v/>
       </c>
       <c r="C24" t="str">
-        <v>07-11-2025</v>
+        <v>07-11-2024</v>
       </c>
       <c r="D24" t="str">
         <v>BankniftyCE</v>
@@ -1512,7 +1512,7 @@
         <v>-1751</v>
       </c>
       <c r="K24">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L24" t="str">
         <v>Yes</v>
@@ -1535,7 +1535,7 @@
         <v/>
       </c>
       <c r="C25" t="str">
-        <v>10-11-2025</v>
+        <v>10-11-2024</v>
       </c>
       <c r="D25" t="str">
         <v>NiftyCE</v>
@@ -1559,7 +1559,7 @@
         <v>-3788</v>
       </c>
       <c r="K25">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L25" t="str">
         <v>Yes</v>
@@ -1582,7 +1582,7 @@
         <v/>
       </c>
       <c r="C26" t="str">
-        <v>11-11-2025</v>
+        <v>11-11-2024</v>
       </c>
       <c r="D26" t="str">
         <v>Sensex PE</v>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
       <c r="K26">
-        <v>-40</v>
+        <v>40</v>
       </c>
       <c r="L26" t="str">
         <v>Yes</v>
@@ -1629,7 +1629,7 @@
         <v/>
       </c>
       <c r="C27" t="str">
-        <v>12-11-2025</v>
+        <v>12-11-2024</v>
       </c>
       <c r="D27" t="str">
         <v>NiftyCE</v>
@@ -1653,7 +1653,7 @@
         <v>-2940</v>
       </c>
       <c r="K27">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L27" t="str">
         <v>Yes</v>
@@ -1676,7 +1676,7 @@
         <v/>
       </c>
       <c r="C28" t="str">
-        <v>12-11-2025</v>
+        <v>12-11-2024</v>
       </c>
       <c r="D28" t="str">
         <v>NiftyCE</v>
@@ -1700,7 +1700,7 @@
         <v>-3383</v>
       </c>
       <c r="K28">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L28" t="str">
         <v>Yes</v>
@@ -1723,7 +1723,7 @@
         <v/>
       </c>
       <c r="C29" t="str">
-        <v>13-11-2025</v>
+        <v>13-11-2024</v>
       </c>
       <c r="D29" t="str">
         <v>NiftyCE</v>
@@ -1747,7 +1747,7 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L29" t="str">
         <v>Yes</v>
@@ -1770,7 +1770,7 @@
         <v/>
       </c>
       <c r="C30" t="str">
-        <v>14-11-2025</v>
+        <v>14-11-2024</v>
       </c>
       <c r="D30" t="str">
         <v>Sensex PE</v>
@@ -1794,7 +1794,7 @@
         <v>-4144</v>
       </c>
       <c r="K30">
-        <v>-40</v>
+        <v>40</v>
       </c>
       <c r="L30" t="str">
         <v>Yes</v>
@@ -1817,7 +1817,7 @@
         <v/>
       </c>
       <c r="C31" t="str">
-        <v>17-11-2025</v>
+        <v>17-11-2024</v>
       </c>
       <c r="D31" t="str">
         <v>BankniftyCE</v>
@@ -1841,7 +1841,7 @@
         <v>0</v>
       </c>
       <c r="K31">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L31" t="str">
         <v>Yes</v>
@@ -1864,7 +1864,7 @@
         <v/>
       </c>
       <c r="C32" t="str">
-        <v>19-11-2025</v>
+        <v>19-11-2024</v>
       </c>
       <c r="D32" t="str">
         <v>BankniftyCE</v>
@@ -1888,7 +1888,7 @@
         <v>-739</v>
       </c>
       <c r="K32">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L32" t="str">
         <v>Yes</v>
@@ -1911,7 +1911,7 @@
         <v/>
       </c>
       <c r="C33" t="str">
-        <v>20-11-2025</v>
+        <v>20-11-2024</v>
       </c>
       <c r="D33" t="str">
         <v>Sensex CE</v>
@@ -1935,7 +1935,7 @@
         <v>-3002</v>
       </c>
       <c r="K33">
-        <v>-40</v>
+        <v>40</v>
       </c>
       <c r="L33" t="str">
         <v>Yes</v>
@@ -1958,7 +1958,7 @@
         <v/>
       </c>
       <c r="C34" t="str">
-        <v>21-11-2025</v>
+        <v>21-11-2024</v>
       </c>
       <c r="D34" t="str">
         <v>BankniftyPE</v>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="K34">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L34" t="str">
         <v>Yes</v>
@@ -2005,7 +2005,7 @@
         <v/>
       </c>
       <c r="C35" t="str">
-        <v>24-11-2025</v>
+        <v>24-11-2024</v>
       </c>
       <c r="D35" t="str">
         <v>BankniftyCE</v>
@@ -2029,7 +2029,7 @@
         <v>0</v>
       </c>
       <c r="K35">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L35" t="str">
         <v>Yes</v>
@@ -2052,7 +2052,7 @@
         <v/>
       </c>
       <c r="C36" t="str">
-        <v>24-11-2025</v>
+        <v>24-11-2024</v>
       </c>
       <c r="D36" t="str">
         <v>BankniftyPE</v>
@@ -2076,7 +2076,7 @@
         <v>0</v>
       </c>
       <c r="K36">
-        <v>-54</v>
+        <v>54</v>
       </c>
       <c r="L36" t="str">
         <v>Yes</v>
@@ -2099,7 +2099,7 @@
         <v/>
       </c>
       <c r="C37" t="str">
-        <v>26-11-2025</v>
+        <v>26-11-2024</v>
       </c>
       <c r="D37" t="str">
         <v>NiftyCE</v>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="K37">
-        <v>-216</v>
+        <v>216</v>
       </c>
       <c r="L37" t="str">
         <v>No</v>
@@ -2146,7 +2146,7 @@
         <v/>
       </c>
       <c r="C38" t="str">
-        <v>03-12-2025</v>
+        <v>03-12-2024</v>
       </c>
       <c r="D38" t="str">
         <v>NiftyPE</v>
@@ -2170,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="K38">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L38" t="str">
         <v>Yes</v>
@@ -2193,7 +2193,7 @@
         <v/>
       </c>
       <c r="C39" t="str">
-        <v>03-12-2025</v>
+        <v>03-12-2024</v>
       </c>
       <c r="D39" t="str">
         <v>BankniftyPE</v>
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="K39">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L39" t="str">
         <v>Yes</v>
@@ -2240,7 +2240,7 @@
         <v/>
       </c>
       <c r="C40" t="str">
-        <v>05-12-2025</v>
+        <v>05-12-2024</v>
       </c>
       <c r="D40" t="str">
         <v>NiftyCE</v>
@@ -2264,7 +2264,7 @@
         <v>-3004</v>
       </c>
       <c r="K40">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L40" t="str">
         <v>yes</v>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="C41" t="str">
-        <v>05-12-2025</v>
+        <v>05-12-2024</v>
       </c>
       <c r="D41" t="str">
         <v>BankniftyCE</v>
@@ -2311,7 +2311,7 @@
         <v>-2156</v>
       </c>
       <c r="K41">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L41" t="str">
         <v>Yes</v>
@@ -2334,7 +2334,7 @@
         <v/>
       </c>
       <c r="C42" t="str">
-        <v>10-12-2025</v>
+        <v>10-12-2024</v>
       </c>
       <c r="D42" t="str">
         <v>NiftyCE</v>
@@ -2358,7 +2358,7 @@
         <v>-1069</v>
       </c>
       <c r="K42">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L42" t="str">
         <v>Yes</v>
@@ -2381,7 +2381,7 @@
         <v/>
       </c>
       <c r="C43" t="str">
-        <v>11-12-2025</v>
+        <v>11-12-2024</v>
       </c>
       <c r="D43" t="str">
         <v>BankniftyCE</v>
@@ -2405,7 +2405,7 @@
         <v>-1936</v>
       </c>
       <c r="K43">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L43" t="str">
         <v>Yes</v>
@@ -2428,7 +2428,7 @@
         <v/>
       </c>
       <c r="C44" t="str">
-        <v>12-12-2025</v>
+        <v>12-12-2024</v>
       </c>
       <c r="D44" t="str">
         <v>Sensex CE</v>
@@ -2452,7 +2452,7 @@
         <v>-1901</v>
       </c>
       <c r="K44">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L44" t="str">
         <v>Yes</v>
@@ -2475,7 +2475,7 @@
         <v/>
       </c>
       <c r="C45" t="str">
-        <v>15-12-2025</v>
+        <v>15-12-2024</v>
       </c>
       <c r="D45" t="str">
         <v>NiftyPE</v>
@@ -2499,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="K45">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L45" t="str">
         <v>Yes</v>
@@ -2522,7 +2522,7 @@
         <v/>
       </c>
       <c r="C46" t="str">
-        <v>16-12-2025</v>
+        <v>16-12-2024</v>
       </c>
       <c r="D46" t="str">
         <v>Sensex PE</v>
@@ -2569,7 +2569,7 @@
         <v/>
       </c>
       <c r="C47" t="str">
-        <v>16-12-2025</v>
+        <v>16-12-2024</v>
       </c>
       <c r="D47" t="str">
         <v>NiftyPE</v>
@@ -2593,7 +2593,7 @@
         <v>-1028</v>
       </c>
       <c r="K47">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L47" t="str">
         <v>Yes</v>
@@ -2616,7 +2616,7 @@
         <v/>
       </c>
       <c r="C48" t="str">
-        <v>18-12-2025</v>
+        <v>18-12-2024</v>
       </c>
       <c r="D48" t="str">
         <v>NiftyPE</v>
@@ -2640,7 +2640,7 @@
         <v>0</v>
       </c>
       <c r="K48">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L48" t="str">
         <v>Yes</v>
@@ -2663,7 +2663,7 @@
         <v/>
       </c>
       <c r="C49" t="str">
-        <v>19-12-2025</v>
+        <v>19-12-2024</v>
       </c>
       <c r="D49" t="str">
         <v>NiftyCE</v>
@@ -2687,7 +2687,7 @@
         <v>-990</v>
       </c>
       <c r="K49">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L49" t="str">
         <v>Yes</v>
@@ -2710,7 +2710,7 @@
         <v/>
       </c>
       <c r="C50" t="str">
-        <v>19-12-2025</v>
+        <v>19-12-2024</v>
       </c>
       <c r="D50" t="str">
         <v>Sensex CE</v>
@@ -2734,7 +2734,7 @@
         <v>-724</v>
       </c>
       <c r="K50">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L50" t="str">
         <v>Yes</v>
@@ -2757,7 +2757,7 @@
         <v/>
       </c>
       <c r="C51" t="str">
-        <v>22-12-2025</v>
+        <v>22-12-2024</v>
       </c>
       <c r="D51" t="str">
         <v>BankniftyCE</v>
@@ -2781,7 +2781,7 @@
         <v>0</v>
       </c>
       <c r="K51">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L51" t="str">
         <v>Yes</v>
@@ -2804,7 +2804,7 @@
         <v/>
       </c>
       <c r="C52" t="str">
-        <v>22-12-2025</v>
+        <v>22-12-2024</v>
       </c>
       <c r="D52" t="str">
         <v>NiftyCE</v>
@@ -2828,7 +2828,7 @@
         <v>-270</v>
       </c>
       <c r="K52">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L52" t="str">
         <v>Yes</v>
@@ -2851,7 +2851,7 @@
         <v/>
       </c>
       <c r="C53" t="str">
-        <v>22-12-2025</v>
+        <v>22-12-2024</v>
       </c>
       <c r="D53" t="str">
         <v>Sensex CE</v>
@@ -2875,7 +2875,7 @@
         <v>-955</v>
       </c>
       <c r="K53">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L53" t="str">
         <v>Yes</v>
@@ -2898,7 +2898,7 @@
         <v/>
       </c>
       <c r="C54" t="str">
-        <v>24-12-2025</v>
+        <v>24-12-2024</v>
       </c>
       <c r="D54" t="str">
         <v>BankniftyCE</v>
@@ -2922,7 +2922,7 @@
         <v>-518</v>
       </c>
       <c r="K54">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L54" t="str">
         <v>Yes</v>
@@ -2945,7 +2945,7 @@
         <v/>
       </c>
       <c r="C55" t="str">
-        <v>24-12-2025</v>
+        <v>24-12-2024</v>
       </c>
       <c r="D55" t="str">
         <v>BankniftyPE</v>
@@ -2969,7 +2969,7 @@
         <v>0</v>
       </c>
       <c r="K55">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L55" t="str">
         <v>Yes</v>
@@ -2992,7 +2992,7 @@
         <v/>
       </c>
       <c r="C56" t="str">
-        <v>24-12-2025</v>
+        <v>24-12-2024</v>
       </c>
       <c r="D56" t="str">
         <v>NiftyPE</v>
@@ -3016,7 +3016,7 @@
         <v>-1193</v>
       </c>
       <c r="K56">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L56" t="str">
         <v>Yes</v>
@@ -3039,7 +3039,7 @@
         <v/>
       </c>
       <c r="C57" t="str">
-        <v>26-12-2025</v>
+        <v>26-12-2024</v>
       </c>
       <c r="D57" t="str">
         <v>BankniftyPE</v>
@@ -3063,7 +3063,7 @@
         <v>-406</v>
       </c>
       <c r="K57">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L57" t="str">
         <v>Yes</v>
@@ -3086,7 +3086,7 @@
         <v/>
       </c>
       <c r="C58" t="str">
-        <v>29-12-2025</v>
+        <v>29-12-2024</v>
       </c>
       <c r="D58" t="str">
         <v>BankniftyPE</v>
@@ -3110,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="K58">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L58" t="str">
         <v>Yes</v>
@@ -3133,7 +3133,7 @@
         <v/>
       </c>
       <c r="C59" t="str">
-        <v>29-12-2025</v>
+        <v>29-12-2024</v>
       </c>
       <c r="D59" t="str">
         <v>NiftyPE</v>
@@ -3157,7 +3157,7 @@
         <v>0</v>
       </c>
       <c r="K59">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L59" t="str">
         <v>Yes</v>
@@ -3180,7 +3180,7 @@
         <v/>
       </c>
       <c r="C60" t="str">
-        <v>30-12-2025</v>
+        <v>30-12-2024</v>
       </c>
       <c r="D60" t="str">
         <v>BankniftyPE</v>
@@ -3204,7 +3204,7 @@
         <v>0</v>
       </c>
       <c r="K60">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L60" t="str">
         <v>Yes</v>
@@ -3227,7 +3227,7 @@
         <v/>
       </c>
       <c r="C61" t="str">
-        <v>30-12-2025</v>
+        <v>30-12-2024</v>
       </c>
       <c r="D61" t="str">
         <v>NiftyPE</v>
@@ -3251,7 +3251,7 @@
         <v>-1958</v>
       </c>
       <c r="K61">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L61" t="str">
         <v>Yes</v>
@@ -3274,7 +3274,7 @@
         <v/>
       </c>
       <c r="C62" t="str">
-        <v>30-12-2025</v>
+        <v>30-12-2024</v>
       </c>
       <c r="D62" t="str">
         <v>Sensex PE</v>
@@ -3298,7 +3298,7 @@
         <v>-1747</v>
       </c>
       <c r="K62">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L62" t="str">
         <v>Yes</v>
@@ -3321,7 +3321,7 @@
         <v/>
       </c>
       <c r="C63" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D63" t="str">
         <v>BankniftyCE</v>
@@ -3345,7 +3345,7 @@
         <v>-458</v>
       </c>
       <c r="K63">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L63" t="str">
         <v>Yes</v>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
       <c r="C64" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D64" t="str">
         <v>NiftyCE</v>
@@ -3392,7 +3392,7 @@
         <v>0</v>
       </c>
       <c r="K64">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L64" t="str">
         <v>Yes</v>
@@ -3415,7 +3415,7 @@
         <v/>
       </c>
       <c r="C65" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D65" t="str">
         <v>BankniftyCE</v>
@@ -3439,7 +3439,7 @@
         <v>0</v>
       </c>
       <c r="K65">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L65" t="str">
         <v>Yes</v>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="C66" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D66" t="str">
         <v>Sensex CE</v>
@@ -3486,7 +3486,7 @@
         <v>0</v>
       </c>
       <c r="K66">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L66" t="str">
         <v>Yes</v>
@@ -3509,7 +3509,7 @@
         <v/>
       </c>
       <c r="C67" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D67" t="str">
         <v>Sensex CE</v>
@@ -3533,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="K67">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L67" t="str">
         <v>Yes</v>
@@ -3556,7 +3556,7 @@
         <v/>
       </c>
       <c r="C68" t="str">
-        <v>31-12-2025</v>
+        <v>31-12-2024</v>
       </c>
       <c r="D68" t="str">
         <v>Sensex CE</v>
@@ -3580,7 +3580,7 @@
         <v>-136</v>
       </c>
       <c r="K68">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L68" t="str">
         <v>Yes</v>
@@ -3603,7 +3603,7 @@
         <v/>
       </c>
       <c r="C69" t="str">
-        <v>02-01-2026</v>
+        <v>02-01-2025</v>
       </c>
       <c r="D69" t="str">
         <v>NiftyCE</v>
@@ -3627,7 +3627,7 @@
         <v>0</v>
       </c>
       <c r="K69">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L69" t="str">
         <v>Yes</v>
@@ -3650,7 +3650,7 @@
         <v/>
       </c>
       <c r="C70" t="str">
-        <v>02-01-2026</v>
+        <v>02-01-2025</v>
       </c>
       <c r="D70" t="str">
         <v>Sensex CE</v>
@@ -3674,7 +3674,7 @@
         <v>-99</v>
       </c>
       <c r="K70">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L70" t="str">
         <v>Yes</v>
@@ -3697,7 +3697,7 @@
         <v/>
       </c>
       <c r="C71" t="str">
-        <v>02-01-2026</v>
+        <v>02-01-2025</v>
       </c>
       <c r="D71" t="str">
         <v>Sensex CE</v>
@@ -3721,7 +3721,7 @@
         <v>-641</v>
       </c>
       <c r="K71">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L71" t="str">
         <v>Yes</v>
@@ -3744,7 +3744,7 @@
         <v/>
       </c>
       <c r="C72" t="str">
-        <v>05-01-2026</v>
+        <v>05-01-2025</v>
       </c>
       <c r="D72" t="str">
         <v>NiftyPE</v>
@@ -3768,7 +3768,7 @@
         <v>-488</v>
       </c>
       <c r="K72">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L72" t="str">
         <v>Yes</v>
@@ -3791,7 +3791,7 @@
         <v/>
       </c>
       <c r="C73" t="str">
-        <v>06-01-2026</v>
+        <v>06-01-2025</v>
       </c>
       <c r="D73" t="str">
         <v>Sensex PE</v>
@@ -3815,7 +3815,7 @@
         <v>-1945</v>
       </c>
       <c r="K73">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L73" t="str">
         <v>Yes</v>
@@ -3838,7 +3838,7 @@
         <v/>
       </c>
       <c r="C74" t="str">
-        <v>07-01-2026</v>
+        <v>07-01-2025</v>
       </c>
       <c r="D74" t="str">
         <v>BankniftyPE</v>
@@ -3862,7 +3862,7 @@
         <v>-842</v>
       </c>
       <c r="K74">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L74" t="str">
         <v>Yes</v>
@@ -3885,7 +3885,7 @@
         <v/>
       </c>
       <c r="C75" t="str">
-        <v>08-01-2026</v>
+        <v>08-01-2025</v>
       </c>
       <c r="D75" t="str">
         <v>NiftyPE</v>
@@ -3909,7 +3909,7 @@
         <v>-744</v>
       </c>
       <c r="K75">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L75" t="str">
         <v>Yes</v>
@@ -3932,7 +3932,7 @@
         <v/>
       </c>
       <c r="C76" t="str">
-        <v>08-01-2026</v>
+        <v>08-01-2025</v>
       </c>
       <c r="D76" t="str">
         <v>BankniftyPE</v>
@@ -3956,7 +3956,7 @@
         <v>-900</v>
       </c>
       <c r="K76">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L76" t="str">
         <v>Yes</v>
@@ -3979,7 +3979,7 @@
         <v/>
       </c>
       <c r="C77" t="str">
-        <v>09-01-2026</v>
+        <v>09-01-2025</v>
       </c>
       <c r="D77" t="str">
         <v>NiftyPE</v>
@@ -4003,7 +4003,7 @@
         <v>0</v>
       </c>
       <c r="K77">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L77" t="str">
         <v>Yes</v>
@@ -4026,7 +4026,7 @@
         <v/>
       </c>
       <c r="C78" t="str">
-        <v>09-01-2026</v>
+        <v>09-01-2025</v>
       </c>
       <c r="D78" t="str">
         <v>BankniftyPE</v>
@@ -4050,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="K78">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L78" t="str">
         <v>Yes</v>
@@ -4073,7 +4073,7 @@
         <v/>
       </c>
       <c r="C79" t="str">
-        <v>12-01-2026</v>
+        <v>12-01-2025</v>
       </c>
       <c r="D79" t="str">
         <v>NiftyPE</v>
@@ -4097,7 +4097,7 @@
         <v>-1723</v>
       </c>
       <c r="K79">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L79" t="str">
         <v>Yes</v>
@@ -4120,7 +4120,7 @@
         <v/>
       </c>
       <c r="C80" t="str">
-        <v>13-01-2026</v>
+        <v>13-01-2025</v>
       </c>
       <c r="D80" t="str">
         <v>NiftyPE</v>
@@ -4144,7 +4144,7 @@
         <v>0</v>
       </c>
       <c r="K80">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L80" t="str">
         <v>Yes</v>
@@ -4167,7 +4167,7 @@
         <v/>
       </c>
       <c r="C81" t="str">
-        <v>13-01-2026</v>
+        <v>13-01-2025</v>
       </c>
       <c r="D81" t="str">
         <v>BankniftyPE</v>
@@ -4191,7 +4191,7 @@
         <v>0</v>
       </c>
       <c r="K81">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L81" t="str">
         <v>Yes</v>
@@ -4214,7 +4214,7 @@
         <v/>
       </c>
       <c r="C82" t="str">
-        <v>14-01-2026</v>
+        <v>14-01-2025</v>
       </c>
       <c r="D82" t="str">
         <v>Sensex PE</v>
@@ -4238,7 +4238,7 @@
         <v>0</v>
       </c>
       <c r="K82">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L82" t="str">
         <v>Yes</v>
@@ -4261,7 +4261,7 @@
         <v/>
       </c>
       <c r="C83" t="str">
-        <v>16-01-2026</v>
+        <v>16-01-2025</v>
       </c>
       <c r="D83" t="str">
         <v>BankniftyCE</v>
@@ -4285,7 +4285,7 @@
         <v>0</v>
       </c>
       <c r="K83">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L83" t="str">
         <v>Yes</v>
@@ -4308,7 +4308,7 @@
         <v/>
       </c>
       <c r="C84" t="str">
-        <v>16-01-2026</v>
+        <v>16-01-2025</v>
       </c>
       <c r="D84" t="str">
         <v>Sensex CE</v>
@@ -4332,7 +4332,7 @@
         <v>0</v>
       </c>
       <c r="K84">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L84" t="str">
         <v>Yes</v>
@@ -4355,7 +4355,7 @@
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>19-01-2026</v>
+        <v>19-01-2025</v>
       </c>
       <c r="D85" t="str">
         <v>Sensex PE</v>
@@ -4379,7 +4379,7 @@
         <v>0</v>
       </c>
       <c r="K85">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L85" t="str">
         <v>Yes</v>
@@ -4402,7 +4402,7 @@
         <v/>
       </c>
       <c r="C86" t="str">
-        <v>19-01-2026</v>
+        <v>19-01-2025</v>
       </c>
       <c r="D86" t="str">
         <v>BankniftyPE</v>
@@ -4426,7 +4426,7 @@
         <v>0</v>
       </c>
       <c r="K86">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L86" t="str">
         <v>No</v>
@@ -4449,7 +4449,7 @@
         <v/>
       </c>
       <c r="C87" t="str">
-        <v>20-01-2026</v>
+        <v>20-01-2025</v>
       </c>
       <c r="D87" t="str">
         <v>Sensex PE</v>
@@ -4473,7 +4473,7 @@
         <v>0</v>
       </c>
       <c r="K87">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L87" t="str">
         <v>Yes</v>
@@ -4496,7 +4496,7 @@
         <v/>
       </c>
       <c r="C88" t="str">
-        <v>21-01-2026</v>
+        <v>21-01-2025</v>
       </c>
       <c r="D88" t="str">
         <v>BankniftyPE</v>
@@ -4520,7 +4520,7 @@
         <v>0</v>
       </c>
       <c r="K88">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L88" t="str">
         <v>No</v>
@@ -4543,7 +4543,7 @@
         <v/>
       </c>
       <c r="C89" t="str">
-        <v>22-01-2026</v>
+        <v>22-01-2025</v>
       </c>
       <c r="D89" t="str">
         <v>BankniftyCE</v>
@@ -4567,7 +4567,7 @@
         <v>0</v>
       </c>
       <c r="K89">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L89" t="str">
         <v>No</v>
@@ -4590,7 +4590,7 @@
         <v/>
       </c>
       <c r="C90" t="str">
-        <v>22-01-2026</v>
+        <v>22-01-2025</v>
       </c>
       <c r="D90" t="str">
         <v>NiftyCE</v>
@@ -4614,7 +4614,7 @@
         <v>0</v>
       </c>
       <c r="K90">
-        <v>-26</v>
+        <v>26</v>
       </c>
       <c r="L90" t="str">
         <v>No</v>
@@ -4637,7 +4637,7 @@
         <v/>
       </c>
       <c r="C91" t="str">
-        <v>22-01-2026</v>
+        <v>22-01-2025</v>
       </c>
       <c r="D91" t="str">
         <v>Sensex CE</v>
@@ -4661,7 +4661,7 @@
         <v>0</v>
       </c>
       <c r="K91">
-        <v>-24</v>
+        <v>24</v>
       </c>
       <c r="L91" t="str">
         <v>No</v>
@@ -4684,7 +4684,7 @@
         <v/>
       </c>
       <c r="C92" t="str">
-        <v>23-01-2026</v>
+        <v>23-01-2025</v>
       </c>
       <c r="D92" t="str">
         <v>Sensex PE</v>
@@ -4708,7 +4708,7 @@
         <v>-353</v>
       </c>
       <c r="K92">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L92" t="str">
         <v>Yes</v>
@@ -4731,7 +4731,7 @@
         <v/>
       </c>
       <c r="C93" t="str">
-        <v>23-01-2026</v>
+        <v>23-01-2025</v>
       </c>
       <c r="D93" t="str">
         <v>NiftyPE</v>
@@ -4755,7 +4755,7 @@
         <v>0</v>
       </c>
       <c r="K93">
-        <v>-105</v>
+        <v>105</v>
       </c>
       <c r="L93" t="str">
         <v>No</v>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="C94" t="str">
-        <v>23-01-2026</v>
+        <v>23-01-2025</v>
       </c>
       <c r="D94" t="str">
         <v>BankniftyPE</v>
@@ -4802,7 +4802,7 @@
         <v>0</v>
       </c>
       <c r="K94">
-        <v>-80</v>
+        <v>80</v>
       </c>
       <c r="L94" t="str">
         <v>Yes</v>
@@ -4825,7 +4825,7 @@
         <v/>
       </c>
       <c r="C95" t="str">
-        <v>29-01-2026</v>
+        <v>29-01-2025</v>
       </c>
       <c r="D95" t="str">
         <v>Sensex PE</v>
@@ -4849,7 +4849,7 @@
         <v>-1886</v>
       </c>
       <c r="K95">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L95" t="str">
         <v>Yes</v>
@@ -4872,7 +4872,7 @@
         <v/>
       </c>
       <c r="C96" t="str">
-        <v>30-01-2026</v>
+        <v>30-01-2025</v>
       </c>
       <c r="D96" t="str">
         <v>BankniftyPE</v>
@@ -4896,7 +4896,7 @@
         <v>-454</v>
       </c>
       <c r="K96">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L96" t="str">
         <v>Yes</v>
@@ -4919,7 +4919,7 @@
         <v/>
       </c>
       <c r="C97" t="str">
-        <v>05-02-2026</v>
+        <v>05-02-2025</v>
       </c>
       <c r="D97" t="str">
         <v>NiftyPE</v>
@@ -4943,7 +4943,7 @@
         <v>0</v>
       </c>
       <c r="K97">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L97" t="str">
         <v>Yes</v>
@@ -4966,7 +4966,7 @@
         <v/>
       </c>
       <c r="C98" t="str">
-        <v>05-02-2026</v>
+        <v>05-02-2025</v>
       </c>
       <c r="D98" t="str">
         <v>Sensex PE</v>
@@ -4990,7 +4990,7 @@
         <v>0</v>
       </c>
       <c r="K98">
-        <v>-22</v>
+        <v>22</v>
       </c>
       <c r="L98" t="str">
         <v>Yes</v>
@@ -5013,7 +5013,7 @@
         <v/>
       </c>
       <c r="C99" t="str">
-        <v>06-02-2026</v>
+        <v>06-02-2025</v>
       </c>
       <c r="D99" t="str">
         <v>Sensex PE</v>
@@ -5037,7 +5037,7 @@
         <v>-1043</v>
       </c>
       <c r="K99">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L99" t="str">
         <v>No</v>
@@ -5060,7 +5060,7 @@
         <v/>
       </c>
       <c r="C100" t="str">
-        <v>09-02-2026</v>
+        <v>09-02-2025</v>
       </c>
       <c r="D100" t="str">
         <v>NiftyCE</v>
@@ -5084,7 +5084,7 @@
         <v>0</v>
       </c>
       <c r="K100">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L100" t="str">
         <v>Yes</v>
@@ -5107,7 +5107,7 @@
         <v/>
       </c>
       <c r="C101" t="str">
-        <v>09-02-2026</v>
+        <v>09-02-2025</v>
       </c>
       <c r="D101" t="str">
         <v>BankniftyCE</v>
@@ -5131,7 +5131,7 @@
         <v>-431</v>
       </c>
       <c r="K101">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L101" t="str">
         <v>No</v>
@@ -5154,7 +5154,7 @@
         <v/>
       </c>
       <c r="C102" t="str">
-        <v>10-02-2026</v>
+        <v>10-02-2025</v>
       </c>
       <c r="D102" t="str">
         <v>NiftyCE</v>
@@ -5178,7 +5178,7 @@
         <v>0</v>
       </c>
       <c r="K102">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L102" t="str">
         <v>Yes</v>
@@ -5201,7 +5201,7 @@
         <v/>
       </c>
       <c r="C103" t="str">
-        <v>10-02-2026</v>
+        <v>10-02-2025</v>
       </c>
       <c r="D103" t="str">
         <v>Sensex CE</v>
@@ -5225,7 +5225,7 @@
         <v>0</v>
       </c>
       <c r="K103">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L103" t="str">
         <v>Yes</v>
@@ -5248,7 +5248,7 @@
         <v/>
       </c>
       <c r="C104" t="str">
-        <v>10-02-2026</v>
+        <v>10-02-2025</v>
       </c>
       <c r="D104" t="str">
         <v>BankniftyPE</v>
@@ -5272,7 +5272,7 @@
         <v>0</v>
       </c>
       <c r="K104">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L104" t="str">
         <v>Yes</v>
@@ -5295,7 +5295,7 @@
         <v/>
       </c>
       <c r="C105" t="str">
-        <v>11-02-2026</v>
+        <v>11-02-2025</v>
       </c>
       <c r="D105" t="str">
         <v>BankniftyCE</v>
@@ -5319,7 +5319,7 @@
         <v>-1551</v>
       </c>
       <c r="K105">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L105" t="str">
         <v>No</v>
@@ -5342,7 +5342,7 @@
         <v/>
       </c>
       <c r="C106" t="str">
-        <v>12-02-2026</v>
+        <v>12-02-2025</v>
       </c>
       <c r="D106" t="str">
         <v>Sensex PE</v>
@@ -5366,7 +5366,7 @@
         <v>0</v>
       </c>
       <c r="K106">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L106" t="str">
         <v>Yes</v>
@@ -5389,7 +5389,7 @@
         <v/>
       </c>
       <c r="C107" t="str">
-        <v>12-02-2026</v>
+        <v>12-02-2025</v>
       </c>
       <c r="D107" t="str">
         <v>BankniftyPE</v>
@@ -5413,7 +5413,7 @@
         <v>0</v>
       </c>
       <c r="K107">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L107" t="str">
         <v>Yes</v>
@@ -5436,7 +5436,7 @@
         <v/>
       </c>
       <c r="C108" t="str">
-        <v>13-02-2026</v>
+        <v>13-02-2025</v>
       </c>
       <c r="D108" t="str">
         <v>Sensex PE</v>
@@ -5460,7 +5460,7 @@
         <v>0</v>
       </c>
       <c r="K108">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L108" t="str">
         <v>Yes</v>
@@ -5483,7 +5483,7 @@
         <v/>
       </c>
       <c r="C109" t="str">
-        <v>18-02-2026</v>
+        <v>18-02-2025</v>
       </c>
       <c r="D109" t="str">
         <v>Sensex PE</v>
@@ -5507,7 +5507,7 @@
         <v>-2007</v>
       </c>
       <c r="K109">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="L109" t="str">
         <v>Yes</v>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
       <c r="C110" t="str">
-        <v>18-02-2026</v>
+        <v>18-02-2025</v>
       </c>
       <c r="D110" t="str">
         <v>BankniftyCE</v>
@@ -5554,7 +5554,7 @@
         <v>0</v>
       </c>
       <c r="K110">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L110" t="str">
         <v>No</v>
@@ -5577,7 +5577,7 @@
         <v/>
       </c>
       <c r="C111" t="str">
-        <v>19-02-2026</v>
+        <v>19-02-2025</v>
       </c>
       <c r="D111" t="str">
         <v>Sensex PE</v>
@@ -5601,7 +5601,7 @@
         <v>0</v>
       </c>
       <c r="K111">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L111" t="str">
         <v>Yes</v>
@@ -5624,7 +5624,7 @@
         <v/>
       </c>
       <c r="C112" t="str">
-        <v>20-02-2026</v>
+        <v>20-02-2025</v>
       </c>
       <c r="D112" t="str">
         <v>BankniftyCE</v>
@@ -5648,7 +5648,7 @@
         <v>-1649</v>
       </c>
       <c r="K112">
-        <v>-28</v>
+        <v>28</v>
       </c>
       <c r="L112" t="str">
         <v>Yes</v>
@@ -5671,7 +5671,7 @@
         <v/>
       </c>
       <c r="C113" t="str">
-        <v>24-02-2026</v>
+        <v>24-02-2025</v>
       </c>
       <c r="D113" t="str">
         <v>Sensex PE</v>
@@ -5695,7 +5695,7 @@
         <v>0</v>
       </c>
       <c r="K113">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L113" t="str">
         <v>Yes</v>
@@ -5718,7 +5718,7 @@
         <v/>
       </c>
       <c r="C114" t="str">
-        <v>24-02-2026</v>
+        <v>24-02-2025</v>
       </c>
       <c r="D114" t="str">
         <v>NiftyPE</v>
@@ -5742,7 +5742,7 @@
         <v>0</v>
       </c>
       <c r="K114">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L114" t="str">
         <v>Yes</v>
@@ -5765,7 +5765,7 @@
         <v/>
       </c>
       <c r="C115" t="str">
-        <v>25-02-2026</v>
+        <v>25-02-2025</v>
       </c>
       <c r="D115" t="str">
         <v>NiftyCE</v>
@@ -5789,7 +5789,7 @@
         <v>0</v>
       </c>
       <c r="K115">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L115" t="str">
         <v>Yes</v>
@@ -5812,7 +5812,7 @@
         <v/>
       </c>
       <c r="C116" t="str">
-        <v>25-02-2026</v>
+        <v>25-02-2025</v>
       </c>
       <c r="D116" t="str">
         <v>NiftyCE</v>
@@ -5836,7 +5836,7 @@
         <v>-1342</v>
       </c>
       <c r="K116">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L116" t="str">
         <v>Yes</v>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="C117" t="str">
-        <v>25-02-2026</v>
+        <v>25-02-2025</v>
       </c>
       <c r="D117" t="str">
         <v>NiftyPE</v>
@@ -5883,7 +5883,7 @@
         <v>0</v>
       </c>
       <c r="K117">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L117" t="str">
         <v>Yes</v>
@@ -5906,7 +5906,7 @@
         <v/>
       </c>
       <c r="C118" t="str">
-        <v>27-02-2026</v>
+        <v>27-02-2025</v>
       </c>
       <c r="D118" t="str">
         <v>NiftyPE</v>
@@ -5930,7 +5930,7 @@
         <v>0</v>
       </c>
       <c r="K118">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L118" t="str">
         <v>Yes</v>
@@ -5953,7 +5953,7 @@
         <v/>
       </c>
       <c r="C119" t="str">
-        <v>02-03-2026</v>
+        <v>02-03-2025</v>
       </c>
       <c r="D119" t="str">
         <v>NiftyPE</v>
@@ -5977,7 +5977,7 @@
         <v>0</v>
       </c>
       <c r="K119">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L119" t="str">
         <v>Yes</v>
@@ -6000,7 +6000,7 @@
         <v/>
       </c>
       <c r="C120" t="str">
-        <v>05-03-2026</v>
+        <v>05-03-2025</v>
       </c>
       <c r="D120" t="str">
         <v>NiftyCE</v>
@@ -6024,7 +6024,7 @@
         <v>0</v>
       </c>
       <c r="K120">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L120" t="str">
         <v>Yes</v>
@@ -6047,7 +6047,7 @@
         <v/>
       </c>
       <c r="C121" t="str">
-        <v>11-03-2026</v>
+        <v>11-03-2025</v>
       </c>
       <c r="D121" t="str">
         <v>BankniftyPE</v>
@@ -6071,7 +6071,7 @@
         <v>0</v>
       </c>
       <c r="K121">
-        <v>-32</v>
+        <v>32</v>
       </c>
       <c r="L121" t="str">
         <v>Yes</v>
@@ -6094,7 +6094,7 @@
         <v/>
       </c>
       <c r="C122" t="str">
-        <v>11-03-2026</v>
+        <v>11-03-2025</v>
       </c>
       <c r="D122" t="str">
         <v>Sensex PE</v>
@@ -6118,7 +6118,7 @@
         <v>0</v>
       </c>
       <c r="K122">
-        <v>-30</v>
+        <v>30</v>
       </c>
       <c r="L122" t="str">
         <v>Yes</v>
@@ -6141,7 +6141,7 @@
         <v/>
       </c>
       <c r="C123" t="str">
-        <v>13-03-2026</v>
+        <v>13-03-2025</v>
       </c>
       <c r="D123" t="str">
         <v>BankniftyPE</v>
@@ -6165,7 +6165,7 @@
         <v>-2076</v>
       </c>
       <c r="K123">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L123" t="str">
         <v>Yes</v>
@@ -6188,7 +6188,7 @@
         <v/>
       </c>
       <c r="C124" t="str">
-        <v>13-03-2026</v>
+        <v>13-03-2025</v>
       </c>
       <c r="D124" t="str">
         <v>Sensex PE</v>
@@ -6212,7 +6212,7 @@
         <v>0</v>
       </c>
       <c r="K124">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L124" t="str">
         <v>Yes</v>
@@ -6235,7 +6235,7 @@
         <v/>
       </c>
       <c r="C125" t="str">
-        <v>18-03-2026</v>
+        <v>18-03-2025</v>
       </c>
       <c r="D125" t="str">
         <v>Sensex CE</v>
@@ -6259,7 +6259,7 @@
         <v>-1471</v>
       </c>
       <c r="K125">
-        <v>-18</v>
+        <v>18</v>
       </c>
       <c r="L125" t="str">
         <v>Yes</v>
@@ -6282,7 +6282,7 @@
         <v/>
       </c>
       <c r="C126" t="str">
-        <v>18-03-2026</v>
+        <v>18-03-2025</v>
       </c>
       <c r="D126" t="str">
         <v>BankniftyCE</v>
@@ -6306,7 +6306,7 @@
         <v>-1766</v>
       </c>
       <c r="K126">
-        <v>-18</v>
+        <v>18</v>
       </c>
       <c r="L126" t="str">
         <v>Yes</v>
@@ -6329,7 +6329,7 @@
         <v/>
       </c>
       <c r="C127" t="str">
-        <v>18-03-2026</v>
+        <v>18-03-2025</v>
       </c>
       <c r="D127" t="str">
         <v>NiftyCE</v>
@@ -6353,7 +6353,7 @@
         <v>-1892</v>
       </c>
       <c r="K127">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L127" t="str">
         <v>Yes</v>
@@ -6376,7 +6376,7 @@
         <v/>
       </c>
       <c r="C128" t="str">
-        <v>19-03-2026</v>
+        <v>19-03-2025</v>
       </c>
       <c r="D128" t="str">
         <v>NiftyPE</v>
@@ -6400,7 +6400,7 @@
         <v>0</v>
       </c>
       <c r="K128">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L128" t="str">
         <v>Yes</v>
@@ -6423,7 +6423,7 @@
         <v/>
       </c>
       <c r="C129" t="str">
-        <v>23-03-2026</v>
+        <v>23-03-2025</v>
       </c>
       <c r="D129" t="str">
         <v>BankniftyPE</v>
@@ -6447,7 +6447,7 @@
         <v>-2081</v>
       </c>
       <c r="K129">
-        <v>-20</v>
+        <v>20</v>
       </c>
       <c r="L129" t="str">
         <v>Yes</v>
@@ -6470,7 +6470,7 @@
         <v/>
       </c>
       <c r="C130" t="str">
-        <v>25-03-2026</v>
+        <v>25-03-2025</v>
       </c>
       <c r="D130" t="str">
         <v>BankniftyCE</v>
@@ -6494,7 +6494,7 @@
         <v>0</v>
       </c>
       <c r="K130">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L130" t="str">
         <v>Yes</v>
@@ -6517,7 +6517,7 @@
         <v/>
       </c>
       <c r="C131" t="str">
-        <v>25-03-2026</v>
+        <v>25-03-2025</v>
       </c>
       <c r="D131" t="str">
         <v>NiftyCE</v>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="K131">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L131" t="str">
         <v>Yes</v>
@@ -6564,7 +6564,7 @@
         <v/>
       </c>
       <c r="C132" t="str">
-        <v>25-03-2026</v>
+        <v>25-03-2025</v>
       </c>
       <c r="D132" t="str">
         <v>Sensex CE</v>
@@ -6588,7 +6588,7 @@
         <v>0</v>
       </c>
       <c r="K132">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L132" t="str">
         <v>Yes</v>
@@ -6611,7 +6611,7 @@
         <v/>
       </c>
       <c r="C133" t="str">
-        <v>27-03-2026</v>
+        <v>27-03-2025</v>
       </c>
       <c r="D133" t="str">
         <v>BankniftyPE</v>
@@ -6635,7 +6635,7 @@
         <v>-2082</v>
       </c>
       <c r="K133">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="L133" t="str">
         <v>Yes</v>
@@ -6658,7 +6658,7 @@
         <v/>
       </c>
       <c r="C134" t="str">
-        <v>08-04-2026</v>
+        <v>08-04-2025</v>
       </c>
       <c r="D134" t="str">
         <v>BankniftyCE</v>
@@ -6682,7 +6682,7 @@
         <v>-3247</v>
       </c>
       <c r="K134">
-        <v>-105</v>
+        <v>105</v>
       </c>
       <c r="L134" t="str">
         <v>Yes</v>
@@ -6705,7 +6705,7 @@
         <v/>
       </c>
       <c r="C135" t="str">
-        <v>10-04-2026</v>
+        <v>10-04-2025</v>
       </c>
       <c r="D135" t="str">
         <v>NiftyCE</v>
@@ -6729,7 +6729,7 @@
         <v>-3790</v>
       </c>
       <c r="K135">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="L135" t="str">
         <v>Yes</v>
@@ -6752,7 +6752,7 @@
         <v/>
       </c>
       <c r="C136" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D136" t="str">
         <v>NiftyCE</v>
@@ -6776,7 +6776,7 @@
         <v>-4817</v>
       </c>
       <c r="K136">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L136" t="str">
         <v>Yes</v>
@@ -6799,7 +6799,7 @@
         <v/>
       </c>
       <c r="C137" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D137" t="str">
         <v>NiftyPE</v>
@@ -6823,7 +6823,7 @@
         <v>0</v>
       </c>
       <c r="K137">
-        <v>-80</v>
+        <v>80</v>
       </c>
       <c r="L137" t="str">
         <v>Yes</v>
@@ -6846,7 +6846,7 @@
         <v/>
       </c>
       <c r="C138" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D138" t="str">
         <v>Sensex CE</v>
@@ -6870,7 +6870,7 @@
         <v>-4684</v>
       </c>
       <c r="K138">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L138" t="str">
         <v>Yes</v>
@@ -6893,7 +6893,7 @@
         <v/>
       </c>
       <c r="C139" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D139" t="str">
         <v>Sensex PE</v>
@@ -6917,7 +6917,7 @@
         <v>0</v>
       </c>
       <c r="K139">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L139" t="str">
         <v>Yes</v>
@@ -6940,7 +6940,7 @@
         <v/>
       </c>
       <c r="C140" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D140" t="str">
         <v>NiftyBullCE</v>
@@ -6964,7 +6964,7 @@
         <v>-2610</v>
       </c>
       <c r="K140">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L140" t="str">
         <v>Yes</v>
@@ -6987,7 +6987,7 @@
         <v/>
       </c>
       <c r="C141" t="str">
-        <v>16-04-2026</v>
+        <v>16-04-2025</v>
       </c>
       <c r="D141" t="str">
         <v>NiftyBullPE</v>
@@ -7011,7 +7011,7 @@
         <v>0</v>
       </c>
       <c r="K141">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L141" t="str">
         <v>Yes</v>
@@ -7034,7 +7034,7 @@
         <v/>
       </c>
       <c r="C142" t="str">
-        <v>17-04-2026</v>
+        <v>17-04-2025</v>
       </c>
       <c r="D142" t="str">
         <v>NiftyCE</v>
@@ -7058,7 +7058,7 @@
         <v>-1573</v>
       </c>
       <c r="K142">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L142" t="str">
         <v>Yes</v>
@@ -7081,7 +7081,7 @@
         <v/>
       </c>
       <c r="C143" t="str">
-        <v>17-04-2026</v>
+        <v>17-04-2025</v>
       </c>
       <c r="D143" t="str">
         <v>NiftyBullCE</v>
@@ -7105,7 +7105,7 @@
         <v>-926</v>
       </c>
       <c r="K143">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L143" t="str">
         <v>Yes</v>
@@ -7128,7 +7128,7 @@
         <v/>
       </c>
       <c r="C144" t="str">
-        <v>20-04-2026</v>
+        <v>20-04-2025</v>
       </c>
       <c r="D144" t="str">
         <v>SensexBullCE</v>
@@ -7152,7 +7152,7 @@
         <v>-168</v>
       </c>
       <c r="K144">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L144" t="str">
         <v>Yes</v>
@@ -7175,7 +7175,7 @@
         <v/>
       </c>
       <c r="C145" t="str">
-        <v>20-04-2026</v>
+        <v>20-04-2025</v>
       </c>
       <c r="D145" t="str">
         <v>NiftyBullPE</v>
@@ -7199,7 +7199,7 @@
         <v>-2285</v>
       </c>
       <c r="K145">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L145" t="str">
         <v>Yes</v>
@@ -7222,7 +7222,7 @@
         <v/>
       </c>
       <c r="C146" t="str">
-        <v>20-04-2026</v>
+        <v>20-04-2025</v>
       </c>
       <c r="D146" t="str">
         <v>BankniftyPE</v>
@@ -7246,7 +7246,7 @@
         <v>0</v>
       </c>
       <c r="K146">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="L146" t="str">
         <v>Yes</v>
@@ -7269,7 +7269,7 @@
         <v/>
       </c>
       <c r="C147" t="str">
-        <v>20-04-2026</v>
+        <v>20-04-2025</v>
       </c>
       <c r="D147" t="str">
         <v>BankniftyCE</v>
@@ -7293,7 +7293,7 @@
         <v>-3345</v>
       </c>
       <c r="K147">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="L147" t="str">
         <v>Yes</v>
@@ -7316,7 +7316,7 @@
         <v/>
       </c>
       <c r="C148" t="str">
-        <v>21-04-2026</v>
+        <v>21-04-2025</v>
       </c>
       <c r="D148" t="str">
         <v>Sensex CE</v>
@@ -7340,7 +7340,7 @@
         <v>0</v>
       </c>
       <c r="K148">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L148" t="str">
         <v>Yes</v>
@@ -7363,7 +7363,7 @@
         <v/>
       </c>
       <c r="C149" t="str">
-        <v>21-04-2026</v>
+        <v>21-04-2025</v>
       </c>
       <c r="D149" t="str">
         <v>SensexBullCE</v>
@@ -7387,7 +7387,7 @@
         <v>-392</v>
       </c>
       <c r="K149">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L149" t="str">
         <v>Yes</v>
@@ -7410,7 +7410,7 @@
         <v/>
       </c>
       <c r="C150" t="str">
-        <v>22-04-2026</v>
+        <v>22-04-2025</v>
       </c>
       <c r="D150" t="str">
         <v>NiftyBullPE</v>
@@ -7434,7 +7434,7 @@
         <v>0</v>
       </c>
       <c r="K150">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L150" t="str">
         <v>Yes</v>
@@ -7457,7 +7457,7 @@
         <v/>
       </c>
       <c r="C151" t="str">
-        <v>22-04-2026</v>
+        <v>22-04-2025</v>
       </c>
       <c r="D151" t="str">
         <v>NiftyPE</v>
@@ -7481,7 +7481,7 @@
         <v>0</v>
       </c>
       <c r="K151">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L151" t="str">
         <v>Yes</v>
@@ -7504,7 +7504,7 @@
         <v/>
       </c>
       <c r="C152" t="str">
-        <v>23-04-2026</v>
+        <v>23-04-2025</v>
       </c>
       <c r="D152" t="str">
         <v>NiftyPE</v>
@@ -7528,7 +7528,7 @@
         <v>-4004</v>
       </c>
       <c r="K152">
-        <v>-94</v>
+        <v>94</v>
       </c>
       <c r="L152" t="str">
         <v>Yes</v>
@@ -7551,7 +7551,7 @@
         <v/>
       </c>
       <c r="C153" t="str">
-        <v>23-04-2026</v>
+        <v>23-04-2025</v>
       </c>
       <c r="D153" t="str">
         <v>NiftyBullPE</v>
@@ -7575,7 +7575,7 @@
         <v>-2278</v>
       </c>
       <c r="K153">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L153" t="str">
         <v>Yes</v>
@@ -7598,7 +7598,7 @@
         <v/>
       </c>
       <c r="C154" t="str">
-        <v>28-04-2026</v>
+        <v>28-04-2025</v>
       </c>
       <c r="D154" t="str">
         <v>NiftyPE</v>
@@ -7622,7 +7622,7 @@
         <v>-4804</v>
       </c>
       <c r="K154">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L154" t="str">
         <v>Yes</v>
@@ -7645,7 +7645,7 @@
         <v/>
       </c>
       <c r="C155" t="str">
-        <v>28-04-2026</v>
+        <v>28-04-2025</v>
       </c>
       <c r="D155" t="str">
         <v>BankniftyPE</v>
@@ -7669,7 +7669,7 @@
         <v>-4189</v>
       </c>
       <c r="K155">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L155" t="str">
         <v>Yes</v>
@@ -7692,7 +7692,7 @@
         <v/>
       </c>
       <c r="C156" t="str">
-        <v>28-04-2026</v>
+        <v>28-04-2025</v>
       </c>
       <c r="D156" t="str">
         <v>NiftyBullPE</v>
@@ -7716,7 +7716,7 @@
         <v>-2301</v>
       </c>
       <c r="K156">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L156" t="str">
         <v>Yes</v>
@@ -7739,7 +7739,7 @@
         <v/>
       </c>
       <c r="C157" t="str">
-        <v>28-04-2026</v>
+        <v>28-04-2025</v>
       </c>
       <c r="D157" t="str">
         <v>SensexBullPE</v>
@@ -7763,7 +7763,7 @@
         <v>-2005</v>
       </c>
       <c r="K157">
-        <v>-91</v>
+        <v>91</v>
       </c>
       <c r="L157" t="str">
         <v>Yes</v>
@@ -7786,7 +7786,7 @@
         <v/>
       </c>
       <c r="C158" t="str">
-        <v>29-04-2026</v>
+        <v>29-04-2025</v>
       </c>
       <c r="D158" t="str">
         <v>NiftyCE</v>
@@ -7810,7 +7810,7 @@
         <v>0</v>
       </c>
       <c r="K158">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L158" t="str">
         <v>Yes</v>
@@ -7833,7 +7833,7 @@
         <v/>
       </c>
       <c r="C159" t="str">
-        <v>29-04-2026</v>
+        <v>29-04-2025</v>
       </c>
       <c r="D159" t="str">
         <v>Sensex CE</v>
@@ -7857,7 +7857,7 @@
         <v>0</v>
       </c>
       <c r="K159">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L159" t="str">
         <v>Yes</v>
@@ -7880,7 +7880,7 @@
         <v/>
       </c>
       <c r="C160" t="str">
-        <v>29-04-2026</v>
+        <v>29-04-2025</v>
       </c>
       <c r="D160" t="str">
         <v>NiftyBullCE</v>
@@ -7904,7 +7904,7 @@
         <v>0</v>
       </c>
       <c r="K160">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L160" t="str">
         <v>Yes</v>
@@ -7927,7 +7927,7 @@
         <v/>
       </c>
       <c r="C161" t="str">
-        <v>29-04-2026</v>
+        <v>29-04-2025</v>
       </c>
       <c r="D161" t="str">
         <v>SensexBullCE</v>
@@ -7951,7 +7951,7 @@
         <v>0</v>
       </c>
       <c r="K161">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L161" t="str">
         <v>Yes</v>
@@ -7974,7 +7974,7 @@
         <v/>
       </c>
       <c r="C162" t="str">
-        <v>30-04-2026</v>
+        <v>30-04-2025</v>
       </c>
       <c r="D162" t="str">
         <v>SensexBullPE</v>
@@ -7998,7 +7998,7 @@
         <v>-2131</v>
       </c>
       <c r="K162">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L162" t="str">
         <v>Yes</v>
@@ -8021,7 +8021,7 @@
         <v/>
       </c>
       <c r="C163" t="str">
-        <v>30-04-2026</v>
+        <v>30-04-2025</v>
       </c>
       <c r="D163" t="str">
         <v>NiftyBullPE</v>
@@ -8045,7 +8045,7 @@
         <v>-2269</v>
       </c>
       <c r="K163">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L163" t="str">
         <v>Yes</v>
@@ -8068,7 +8068,7 @@
         <v/>
       </c>
       <c r="C164" t="str">
-        <v>30-04-2026</v>
+        <v>30-04-2025</v>
       </c>
       <c r="D164" t="str">
         <v>Sensex PE</v>
@@ -8092,7 +8092,7 @@
         <v>-3796</v>
       </c>
       <c r="K164">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L164" t="str">
         <v>Yes</v>
@@ -8115,7 +8115,7 @@
         <v/>
       </c>
       <c r="C165" t="str">
-        <v>30-04-2026</v>
+        <v>30-04-2025</v>
       </c>
       <c r="D165" t="str">
         <v>Sensex PE</v>
@@ -8139,7 +8139,7 @@
         <v>0</v>
       </c>
       <c r="K165">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L165" t="str">
         <v>Yes</v>
@@ -8162,7 +8162,7 @@
         <v/>
       </c>
       <c r="C166" t="str">
-        <v>30-04-2026</v>
+        <v>30-04-2025</v>
       </c>
       <c r="D166" t="str">
         <v>NiftyPE</v>
@@ -8186,7 +8186,7 @@
         <v>-1476</v>
       </c>
       <c r="K166">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L166" t="str">
         <v>Yes</v>
@@ -8209,7 +8209,7 @@
         <v/>
       </c>
       <c r="C167" t="str">
-        <v>04-05-2026</v>
+        <v>04-05-2025</v>
       </c>
       <c r="D167" t="str">
         <v>SensexBullCE</v>
@@ -8233,7 +8233,7 @@
         <v>-2010</v>
       </c>
       <c r="K167">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L167" t="str">
         <v>Yes</v>
@@ -8256,7 +8256,7 @@
         <v/>
       </c>
       <c r="C168" t="str">
-        <v>04-05-2026</v>
+        <v>04-05-2025</v>
       </c>
       <c r="D168" t="str">
         <v>NiftyBullCE</v>
@@ -8280,7 +8280,7 @@
         <v>-2720</v>
       </c>
       <c r="K168">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L168" t="str">
         <v>Yes</v>
@@ -8303,7 +8303,7 @@
         <v/>
       </c>
       <c r="C169" t="str">
-        <v>04-05-2026</v>
+        <v>04-05-2025</v>
       </c>
       <c r="D169" t="str">
         <v>BankniftyPE</v>
@@ -8327,7 +8327,7 @@
         <v>0</v>
       </c>
       <c r="K169">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L169" t="str">
         <v>Yes</v>
@@ -8350,7 +8350,7 @@
         <v/>
       </c>
       <c r="C170" t="str">
-        <v>04-05-2026</v>
+        <v>04-05-2025</v>
       </c>
       <c r="D170" t="str">
         <v>BankniftyCE</v>
@@ -8374,7 +8374,7 @@
         <v>-1023</v>
       </c>
       <c r="K170">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L170" t="str">
         <v>Yes</v>
@@ -8397,7 +8397,7 @@
         <v/>
       </c>
       <c r="C171" t="str">
-        <v>05-05-2026</v>
+        <v>05-05-2025</v>
       </c>
       <c r="D171" t="str">
         <v>SensexBullPE</v>
@@ -8421,7 +8421,7 @@
         <v>-2072</v>
       </c>
       <c r="K171">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L171" t="str">
         <v>Yes</v>
@@ -8444,7 +8444,7 @@
         <v/>
       </c>
       <c r="C172" t="str">
-        <v>05-05-2026</v>
+        <v>05-05-2025</v>
       </c>
       <c r="D172" t="str">
         <v>NiftyBullPE</v>
@@ -8468,7 +8468,7 @@
         <v>-2327</v>
       </c>
       <c r="K172">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L172" t="str">
         <v>Yes</v>
@@ -8491,7 +8491,7 @@
         <v/>
       </c>
       <c r="C173" t="str">
-        <v>05-05-2026</v>
+        <v>05-05-2025</v>
       </c>
       <c r="D173" t="str">
         <v>Sensex PE</v>
@@ -8515,7 +8515,7 @@
         <v>-3826</v>
       </c>
       <c r="K173">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L173" t="str">
         <v>Yes</v>
@@ -8538,7 +8538,7 @@
         <v/>
       </c>
       <c r="C174" t="str">
-        <v>05-05-2026</v>
+        <v>05-05-2025</v>
       </c>
       <c r="D174" t="str">
         <v>NiftyPE</v>
@@ -8562,7 +8562,7 @@
         <v>-4583</v>
       </c>
       <c r="K174">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L174" t="str">
         <v>Yes</v>
@@ -8585,7 +8585,7 @@
         <v/>
       </c>
       <c r="C175" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D175" t="str">
         <v>SensexBullCE</v>
@@ -8609,7 +8609,7 @@
         <v>-2018</v>
       </c>
       <c r="K175">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L175" t="str">
         <v>Yes</v>
@@ -8632,7 +8632,7 @@
         <v/>
       </c>
       <c r="C176" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D176" t="str">
         <v>SensexBullPE</v>
@@ -8656,7 +8656,7 @@
         <v>-2015</v>
       </c>
       <c r="K176">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L176" t="str">
         <v>Yes</v>
@@ -8679,7 +8679,7 @@
         <v/>
       </c>
       <c r="C177" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D177" t="str">
         <v>NiftyBullCE</v>
@@ -8703,7 +8703,7 @@
         <v>-1053</v>
       </c>
       <c r="K177">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L177" t="str">
         <v>Yes</v>
@@ -8726,7 +8726,7 @@
         <v/>
       </c>
       <c r="C178" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D178" t="str">
         <v>NiftyBullCE</v>
@@ -8750,7 +8750,7 @@
         <v>0</v>
       </c>
       <c r="K178">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L178" t="str">
         <v>Yes</v>
@@ -8773,7 +8773,7 @@
         <v/>
       </c>
       <c r="C179" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D179" t="str">
         <v>BankniftyCE</v>
@@ -8797,7 +8797,7 @@
         <v>-2816</v>
       </c>
       <c r="K179">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L179" t="str">
         <v>Yes</v>
@@ -8820,7 +8820,7 @@
         <v/>
       </c>
       <c r="C180" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D180" t="str">
         <v>NiftyCE</v>
@@ -8844,7 +8844,7 @@
         <v>-2074</v>
       </c>
       <c r="K180">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L180" t="str">
         <v>Yes</v>
@@ -8867,7 +8867,7 @@
         <v/>
       </c>
       <c r="C181" t="str">
-        <v>06-05-2026</v>
+        <v>06-05-2025</v>
       </c>
       <c r="D181" t="str">
         <v>NiftyCE</v>
@@ -8891,7 +8891,7 @@
         <v>0</v>
       </c>
       <c r="K181">
-        <v>-71</v>
+        <v>71</v>
       </c>
       <c r="L181" t="str">
         <v>Yes</v>
@@ -8914,7 +8914,7 @@
         <v/>
       </c>
       <c r="C182" t="str">
-        <v>08-05-2026</v>
+        <v>08-05-2025</v>
       </c>
       <c r="D182" t="str">
         <v>SensexBullPE</v>
@@ -8938,7 +8938,7 @@
         <v>0</v>
       </c>
       <c r="K182">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L182" t="str">
         <v>Yes</v>
@@ -8961,7 +8961,7 @@
         <v/>
       </c>
       <c r="C183" t="str">
-        <v>08-05-2026</v>
+        <v>08-05-2025</v>
       </c>
       <c r="D183" t="str">
         <v>NiftyBullPE</v>
@@ -8985,7 +8985,7 @@
         <v>0</v>
       </c>
       <c r="K183">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L183" t="str">
         <v>Yes</v>
@@ -9008,7 +9008,7 @@
         <v/>
       </c>
       <c r="C184" t="str">
-        <v>08-05-2026</v>
+        <v>08-05-2025</v>
       </c>
       <c r="D184" t="str">
         <v>BankniftyPE</v>
@@ -9032,7 +9032,7 @@
         <v>0</v>
       </c>
       <c r="K184">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L184" t="str">
         <v>Yes</v>
@@ -9055,7 +9055,7 @@
         <v/>
       </c>
       <c r="C185" t="str">
-        <v>08-05-2026</v>
+        <v>08-05-2025</v>
       </c>
       <c r="D185" t="str">
         <v>Sensex PE</v>
@@ -9079,7 +9079,7 @@
         <v>0</v>
       </c>
       <c r="K185">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L185" t="str">
         <v>Yes</v>
@@ -9102,7 +9102,7 @@
         <v/>
       </c>
       <c r="C186" t="str">
-        <v>08-05-2026</v>
+        <v>08-05-2025</v>
       </c>
       <c r="D186" t="str">
         <v>NiftyPE</v>
@@ -9126,7 +9126,7 @@
         <v>0</v>
       </c>
       <c r="K186">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L186" t="str">
         <v>Yes</v>
@@ -9149,7 +9149,7 @@
         <v/>
       </c>
       <c r="C187" t="str">
-        <v>11-05-2026</v>
+        <v>11-05-2025</v>
       </c>
       <c r="D187" t="str">
         <v>NiftyBullPE</v>
@@ -9173,7 +9173,7 @@
         <v>-2275</v>
       </c>
       <c r="K187">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L187" t="str">
         <v>Yes</v>
@@ -9196,7 +9196,7 @@
         <v/>
       </c>
       <c r="C188" t="str">
-        <v>11-05-2026</v>
+        <v>11-05-2025</v>
       </c>
       <c r="D188" t="str">
         <v>BankniftyPE</v>
@@ -9220,7 +9220,7 @@
         <v>-4175</v>
       </c>
       <c r="K188">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L188" t="str">
         <v>Yes</v>
@@ -9243,7 +9243,7 @@
         <v/>
       </c>
       <c r="C189" t="str">
-        <v>11-05-2026</v>
+        <v>11-05-2025</v>
       </c>
       <c r="D189" t="str">
         <v>Sensex PE</v>
@@ -9267,7 +9267,7 @@
         <v>0</v>
       </c>
       <c r="K189">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L189" t="str">
         <v>Yes</v>
@@ -9290,7 +9290,7 @@
         <v/>
       </c>
       <c r="C190" t="str">
-        <v>11-05-2026</v>
+        <v>11-05-2025</v>
       </c>
       <c r="D190" t="str">
         <v>NiftyPE</v>
@@ -9314,7 +9314,7 @@
         <v>0</v>
       </c>
       <c r="K190">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="L190" t="str">
         <v>Yes</v>
@@ -9337,7 +9337,7 @@
         <v/>
       </c>
       <c r="C191" t="str">
-        <v>12-05-2026</v>
+        <v>12-05-2025</v>
       </c>
       <c r="D191" t="str">
         <v>SensexBullPE</v>
@@ -9361,7 +9361,7 @@
         <v>0</v>
       </c>
       <c r="K191">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L191" t="str">
         <v>Yes</v>
@@ -9384,7 +9384,7 @@
         <v/>
       </c>
       <c r="C192" t="str">
-        <v>12-05-2026</v>
+        <v>12-05-2025</v>
       </c>
       <c r="D192" t="str">
         <v>NiftyBullPE</v>
@@ -9408,7 +9408,7 @@
         <v>0</v>
       </c>
       <c r="K192">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L192" t="str">
         <v>Yes</v>
@@ -9431,7 +9431,7 @@
         <v/>
       </c>
       <c r="C193" t="str">
-        <v>12-05-2026</v>
+        <v>12-05-2025</v>
       </c>
       <c r="D193" t="str">
         <v>NiftyPE</v>
@@ -9455,7 +9455,7 @@
         <v>0</v>
       </c>
       <c r="K193">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="L193" t="str">
         <v>Yes</v>
@@ -9478,7 +9478,7 @@
         <v/>
       </c>
       <c r="C194" t="str">
-        <v>13-05-2026</v>
+        <v>13-05-2025</v>
       </c>
       <c r="D194" t="str">
         <v>SensexBullPE</v>
@@ -9502,7 +9502,7 @@
         <v>-2075</v>
       </c>
       <c r="K194">
-        <v>-85</v>
+        <v>85</v>
       </c>
       <c r="L194" t="str">
         <v>Yes</v>
@@ -9525,7 +9525,7 @@
         <v/>
       </c>
       <c r="C195" t="str">
-        <v>13-05-2026</v>
+        <v>13-05-2025</v>
       </c>
       <c r="D195" t="str">
         <v>NiftyBullPE</v>
@@ -9549,7 +9549,7 @@
         <v>-2106</v>
       </c>
       <c r="K195">
-        <v>-85</v>
+        <v>85</v>
       </c>
       <c r="L195" t="str">
         <v>Yes</v>
@@ -9572,7 +9572,7 @@
         <v/>
       </c>
       <c r="C196" t="str">
-        <v>13-05-2026</v>
+        <v>13-05-2025</v>
       </c>
       <c r="D196" t="str">
         <v>BankniftyPE</v>
@@ -9596,7 +9596,7 @@
         <v>-4047</v>
       </c>
       <c r="K196">
-        <v>-86</v>
+        <v>86</v>
       </c>
       <c r="L196" t="str">
         <v>Yes</v>
@@ -9619,7 +9619,7 @@
         <v/>
       </c>
       <c r="C197" t="str">
-        <v>14-05-2026</v>
+        <v>14-05-2025</v>
       </c>
       <c r="D197" t="str">
         <v>SensexBullCE</v>
@@ -9643,7 +9643,7 @@
         <v>0</v>
       </c>
       <c r="K197">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="L197" t="str">
         <v>Yes</v>
@@ -9666,7 +9666,7 @@
         <v/>
       </c>
       <c r="C198" t="str">
-        <v>14-05-2026</v>
+        <v>14-05-2025</v>
       </c>
       <c r="D198" t="str">
         <v>NiftyBullCE</v>
@@ -9690,7 +9690,7 @@
         <v>0</v>
       </c>
       <c r="K198">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="L198" t="str">
         <v>Yes</v>
@@ -9713,7 +9713,7 @@
         <v/>
       </c>
       <c r="C199" t="str">
-        <v>14-05-2026</v>
+        <v>14-05-2025</v>
       </c>
       <c r="D199" t="str">
         <v>BankniftyCE</v>
@@ -9737,7 +9737,7 @@
         <v>0</v>
       </c>
       <c r="K199">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="L199" t="str">
         <v>Yes</v>
@@ -9760,7 +9760,7 @@
         <v/>
       </c>
       <c r="C200" t="str">
-        <v>14-05-2026</v>
+        <v>14-05-2025</v>
       </c>
       <c r="D200" t="str">
         <v>Sensex CE</v>
@@ -9784,7 +9784,7 @@
         <v>0</v>
       </c>
       <c r="K200">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="L200" t="str">
         <v>Yes</v>
@@ -9807,7 +9807,7 @@
         <v/>
       </c>
       <c r="C201" t="str">
-        <v>14-05-2026</v>
+        <v>14-05-2025</v>
       </c>
       <c r="D201" t="str">
         <v>NiftyCE</v>
@@ -9831,7 +9831,7 @@
         <v>0</v>
       </c>
       <c r="K201">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="L201" t="str">
         <v>Yes</v>
@@ -9854,7 +9854,7 @@
         <v/>
       </c>
       <c r="C202" t="str">
-        <v>18-05-2026</v>
+        <v>18-05-2025</v>
       </c>
       <c r="D202" t="str">
         <v>SensexBullPE</v>
@@ -9878,7 +9878,7 @@
         <v>0</v>
       </c>
       <c r="K202">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L202" t="str">
         <v>Yes</v>
@@ -9901,7 +9901,7 @@
         <v/>
       </c>
       <c r="C203" t="str">
-        <v>18-05-2026</v>
+        <v>18-05-2025</v>
       </c>
       <c r="D203" t="str">
         <v>NiftyBullPE</v>
@@ -9925,7 +9925,7 @@
         <v>0</v>
       </c>
       <c r="K203">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L203" t="str">
         <v>Yes</v>
@@ -9948,7 +9948,7 @@
         <v/>
       </c>
       <c r="C204" t="str">
-        <v>18-05-2026</v>
+        <v>18-05-2025</v>
       </c>
       <c r="D204" t="str">
         <v>Sensex PE</v>
@@ -9972,7 +9972,7 @@
         <v>0</v>
       </c>
       <c r="K204">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L204" t="str">
         <v>Yes</v>
@@ -9995,7 +9995,7 @@
         <v/>
       </c>
       <c r="C205" t="str">
-        <v>18-05-2026</v>
+        <v>18-05-2025</v>
       </c>
       <c r="D205" t="str">
         <v>NiftyPE</v>
@@ -10019,7 +10019,7 @@
         <v>0</v>
       </c>
       <c r="K205">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L205" t="str">
         <v>Yes</v>
@@ -10042,7 +10042,7 @@
         <v/>
       </c>
       <c r="C206" t="str">
-        <v>20-05-2026</v>
+        <v>20-05-2025</v>
       </c>
       <c r="D206" t="str">
         <v>SensexBullPE</v>
@@ -10066,7 +10066,7 @@
         <v>-2000</v>
       </c>
       <c r="K206">
-        <v>-92</v>
+        <v>92</v>
       </c>
       <c r="L206" t="str">
         <v>Yes</v>
@@ -10089,7 +10089,7 @@
         <v/>
       </c>
       <c r="C207" t="str">
-        <v>20-05-2026</v>
+        <v>20-05-2025</v>
       </c>
       <c r="D207" t="str">
         <v>NiftyBullPE</v>
@@ -10113,7 +10113,7 @@
         <v>-1466</v>
       </c>
       <c r="K207">
-        <v>-92</v>
+        <v>92</v>
       </c>
       <c r="L207" t="str">
         <v>Yes</v>
@@ -10136,7 +10136,7 @@
         <v/>
       </c>
       <c r="C208" t="str">
-        <v>20-05-2026</v>
+        <v>20-05-2025</v>
       </c>
       <c r="D208" t="str">
         <v>BankniftyPE</v>
@@ -10160,7 +10160,7 @@
         <v>-3597</v>
       </c>
       <c r="K208">
-        <v>-92</v>
+        <v>92</v>
       </c>
       <c r="L208" t="str">
         <v>Yes</v>
@@ -10183,7 +10183,7 @@
         <v/>
       </c>
       <c r="C209" t="str">
-        <v>20-05-2026</v>
+        <v>20-05-2025</v>
       </c>
       <c r="D209" t="str">
         <v>NiftyPE</v>
@@ -10207,7 +10207,7 @@
         <v>-2496</v>
       </c>
       <c r="K209">
-        <v>-94</v>
+        <v>94</v>
       </c>
       <c r="L209" t="str">
         <v>Yes</v>
@@ -10230,7 +10230,7 @@
         <v/>
       </c>
       <c r="C210" t="str">
-        <v>21-05-2026</v>
+        <v>21-05-2025</v>
       </c>
       <c r="D210" t="str">
         <v>NiftyBullPE</v>
@@ -10254,7 +10254,7 @@
         <v>-2291</v>
       </c>
       <c r="K210">
-        <v>-80</v>
+        <v>80</v>
       </c>
       <c r="L210" t="str">
         <v>Yes</v>
@@ -10277,7 +10277,7 @@
         <v/>
       </c>
       <c r="C211" t="str">
-        <v>22-05-2026</v>
+        <v>22-05-2025</v>
       </c>
       <c r="D211" t="str">
         <v>Sensex CE</v>
@@ -10301,7 +10301,7 @@
         <v>-2648</v>
       </c>
       <c r="K211">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L211" t="str">
         <v>Yes</v>
@@ -10324,7 +10324,7 @@
         <v/>
       </c>
       <c r="C212" t="str">
-        <v>22-05-2026</v>
+        <v>22-05-2025</v>
       </c>
       <c r="D212" t="str">
         <v>BankniftyCE</v>
@@ -10348,7 +10348,7 @@
         <v>-2769</v>
       </c>
       <c r="K212">
-        <v>-98</v>
+        <v>98</v>
       </c>
       <c r="L212" t="str">
         <v>Yes</v>
@@ -10371,7 +10371,7 @@
         <v/>
       </c>
       <c r="C213" t="str">
-        <v>25-05-2026</v>
+        <v>25-05-2025</v>
       </c>
       <c r="D213" t="str">
         <v>NiftyCE</v>
@@ -10395,7 +10395,7 @@
         <v>-3760</v>
       </c>
       <c r="K213">
-        <v>-160</v>
+        <v>160</v>
       </c>
       <c r="L213" t="str">
         <v>Yes</v>
@@ -10418,7 +10418,7 @@
         <v/>
       </c>
       <c r="C214" t="str">
-        <v>25-05-2026</v>
+        <v>25-05-2025</v>
       </c>
       <c r="D214" t="str">
         <v>Sensex CE</v>
@@ -10442,7 +10442,7 @@
         <v>-2578</v>
       </c>
       <c r="K214">
-        <v>-155</v>
+        <v>155</v>
       </c>
       <c r="L214" t="str">
         <v>Yes</v>
@@ -10465,7 +10465,7 @@
         <v/>
       </c>
       <c r="C215" t="str">
-        <v>25-05-2026</v>
+        <v>25-05-2025</v>
       </c>
       <c r="D215" t="str">
         <v>Sensex CE</v>
@@ -10489,7 +10489,7 @@
         <v>-3473</v>
       </c>
       <c r="K215">
-        <v>-154</v>
+        <v>154</v>
       </c>
       <c r="L215" t="str">
         <v>Yes</v>
@@ -10512,7 +10512,7 @@
         <v/>
       </c>
       <c r="C216" t="str">
-        <v>25-05-2026</v>
+        <v>25-05-2025</v>
       </c>
       <c r="D216" t="str">
         <v>BankniftyCE</v>
@@ -10536,7 +10536,7 @@
         <v>-4649</v>
       </c>
       <c r="K216">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="L216" t="str">
         <v>Yes</v>
@@ -10559,7 +10559,7 @@
         <v/>
       </c>
       <c r="C217" t="str">
-        <v>25-05-2026</v>
+        <v>25-05-2025</v>
       </c>
       <c r="D217" t="str">
         <v>BankniftyCE</v>
@@ -10583,7 +10583,7 @@
         <v>0</v>
       </c>
       <c r="K217">
-        <v>-150</v>
+        <v>150</v>
       </c>
       <c r="L217" t="str">
         <v>Yes</v>
@@ -10606,7 +10606,7 @@
         <v/>
       </c>
       <c r="C218" t="str">
-        <v>26-05-2026</v>
+        <v>26-05-2025</v>
       </c>
       <c r="D218" t="str">
         <v>Sensex PE</v>
@@ -10630,7 +10630,7 @@
         <v>-5685</v>
       </c>
       <c r="K218">
-        <v>-146</v>
+        <v>146</v>
       </c>
       <c r="L218" t="str">
         <v>Yes</v>
@@ -10653,7 +10653,7 @@
         <v/>
       </c>
       <c r="C219" t="str">
-        <v>26-05-2026</v>
+        <v>26-05-2025</v>
       </c>
       <c r="D219" t="str">
         <v>NiftyPE</v>
@@ -10677,7 +10677,7 @@
         <v>0</v>
       </c>
       <c r="K219">
-        <v>-146</v>
+        <v>146</v>
       </c>
       <c r="L219" t="str">
         <v>Yes</v>
@@ -10700,7 +10700,7 @@
         <v/>
       </c>
       <c r="C220" t="str">
-        <v>29-05-2026</v>
+        <v>29-05-2025</v>
       </c>
       <c r="D220" t="str">
         <v>Sensex PE</v>
@@ -10724,7 +10724,7 @@
         <v>0</v>
       </c>
       <c r="K220">
-        <v>-61</v>
+        <v>61</v>
       </c>
       <c r="L220" t="str">
         <v>Yes</v>
@@ -10739,56 +10739,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" t="str">
-        <v/>
-      </c>
-      <c r="B221" t="str">
-        <v/>
-      </c>
-      <c r="C221" t="str">
-        <v>01-06-2026</v>
-      </c>
-      <c r="D221" t="str">
-        <v>BankniftyPE</v>
-      </c>
-      <c r="E221">
-        <v>120</v>
-      </c>
-      <c r="F221">
-        <v>522.8</v>
-      </c>
-      <c r="G221">
-        <v>496.85</v>
-      </c>
-      <c r="H221">
-        <v>-25.949999999999932</v>
-      </c>
-      <c r="I221">
-        <v>0</v>
-      </c>
-      <c r="J221">
-        <v>3243.999999999992</v>
-      </c>
-      <c r="K221">
-        <v>130</v>
-      </c>
-      <c r="L221" t="str">
-        <v>YES</v>
-      </c>
-      <c r="M221" t="str">
-        <v/>
-      </c>
-      <c r="N221">
-        <v>-3243.999999999992</v>
-      </c>
-      <c r="O221">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O221"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O220"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>